<commit_message>
v2p1 created and test success
</commit_message>
<xml_diff>
--- a/out/stir_daily_system_wide_with GRAPHS_22Oct25.xlsx
+++ b/out/stir_daily_system_wide_with GRAPHS_22Oct25.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c7d62234183fd3ba/Documents/GitHub/kerbel-long-term-impacts/out/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="8_{3109FC4A-BD15-44FB-B1BB-C01FAB71276C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B51F7A19-4EAD-5856-B5B2-4BA41BA417C6}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="8_{3109FC4A-BD15-44FB-B1BB-C01FAB71276C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{661B7CAB-B345-4CAE-AAAE-F088D9D70E99}"/>
   <bookViews>
-    <workbookView xWindow="-28695" yWindow="2340" windowWidth="28800" windowHeight="13155" xr2:uid="{95A4D3B7-9F89-4514-B226-E93CDF5B25B1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{95A4D3B7-9F89-4514-B226-E93CDF5B25B1}"/>
   </bookViews>
   <sheets>
     <sheet name="stir_daily_system_wide" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Date</t>
   </si>
@@ -98,6 +98,15 @@
   </si>
   <si>
     <t>MT_STIR_Sum_All</t>
+  </si>
+  <si>
+    <t>CT</t>
+  </si>
+  <si>
+    <t>ST</t>
+  </si>
+  <si>
+    <t>MT</t>
   </si>
 </sst>
 </file>
@@ -631,6 +640,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFF9E87F"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -649,10 +663,10 @@
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
+      <c14:style val="101"/>
     </mc:Choice>
     <mc:Fallback>
-      <c:style val="2"/>
+      <c:style val="1"/>
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
@@ -667,49 +681,26 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>stir_daily_system_wide!$U$1</c:f>
+              <c:f>stir_daily_system_wide!$AC$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>CT_STIR_Sum_Year</c:v>
+                  <c:v>CT</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:gradFill rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:schemeClr val="accent1">
-                    <a:lumMod val="110000"/>
-                    <a:satMod val="105000"/>
-                    <a:tint val="67000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:schemeClr val="accent1">
-                    <a:lumMod val="105000"/>
-                    <a:satMod val="103000"/>
-                    <a:tint val="73000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:schemeClr val="accent1">
-                    <a:lumMod val="105000"/>
-                    <a:satMod val="109000"/>
-                    <a:tint val="81000"/>
-                  </a:schemeClr>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000" scaled="0"/>
-            </a:gradFill>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx2">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
               <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:shade val="95000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent1"/>
               </a:solidFill>
-              <a:round/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
@@ -1780,49 +1771,26 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>stir_daily_system_wide!$W$1</c:f>
+              <c:f>stir_daily_system_wide!$AD$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>ST_STIR_Sum_Year</c:v>
+                  <c:v>ST</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:gradFill rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:schemeClr val="accent2">
-                    <a:lumMod val="110000"/>
-                    <a:satMod val="105000"/>
-                    <a:tint val="67000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:schemeClr val="accent2">
-                    <a:lumMod val="105000"/>
-                    <a:satMod val="103000"/>
-                    <a:tint val="73000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:schemeClr val="accent2">
-                    <a:lumMod val="105000"/>
-                    <a:satMod val="109000"/>
-                    <a:tint val="81000"/>
-                  </a:schemeClr>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000" scaled="0"/>
-            </a:gradFill>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="accent5">
+                <a:lumMod val="60000"/>
+                <a:lumOff val="40000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
               <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:shade val="95000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent5"/>
               </a:solidFill>
-              <a:round/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
@@ -2893,49 +2861,27 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>stir_daily_system_wide!$Y$1</c:f>
+              <c:f>stir_daily_system_wide!$AE$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>MT_STIR_Sum_Year</c:v>
+                  <c:v>MT</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:gradFill rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:schemeClr val="accent3">
-                    <a:lumMod val="110000"/>
-                    <a:satMod val="105000"/>
-                    <a:tint val="67000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:schemeClr val="accent3">
-                    <a:lumMod val="105000"/>
-                    <a:satMod val="103000"/>
-                    <a:tint val="73000"/>
-                  </a:schemeClr>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:schemeClr val="accent3">
-                    <a:lumMod val="105000"/>
-                    <a:satMod val="109000"/>
-                    <a:tint val="81000"/>
-                  </a:schemeClr>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000" scaled="0"/>
-            </a:gradFill>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:srgbClr val="F9E87F">
+                <a:alpha val="69804"/>
+              </a:srgbClr>
+            </a:solidFill>
+            <a:ln>
               <a:solidFill>
-                <a:schemeClr val="accent3">
-                  <a:shade val="95000"/>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="75000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:round/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
@@ -4033,14 +3979,19 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="m/d/yyyy" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:numFmt formatCode="m/d/yy;@" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
           <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:noFill/>
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
             <a:round/>
           </a:ln>
           <a:effectLst/>
@@ -4050,16 +4001,13 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="50000"/>
-                    <a:lumOff val="50000"/>
-                  </a:schemeClr>
+                  <a:sysClr val="windowText" lastClr="000000"/>
                 </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
+                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
+                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:defRPr>
             </a:pPr>
             <a:endParaRPr lang="en-US"/>
@@ -4099,16 +4047,13 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                  <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="50000"/>
-                        <a:lumOff val="50000"/>
-                      </a:schemeClr>
+                      <a:sysClr val="windowText" lastClr="000000"/>
                     </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
+                    <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                     <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
+                    <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
@@ -4131,16 +4076,13 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="50000"/>
-                      <a:lumOff val="50000"/>
-                    </a:schemeClr>
+                    <a:sysClr val="windowText" lastClr="000000"/>
                   </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
+                  <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                   <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
+                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 </a:defRPr>
               </a:pPr>
               <a:endParaRPr lang="en-US"/>
@@ -4163,23 +4105,20 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="50000"/>
-                    <a:lumOff val="50000"/>
-                  </a:schemeClr>
+                  <a:sysClr val="windowText" lastClr="000000"/>
                 </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
+                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
+                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:defRPr>
             </a:pPr>
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="1258194463"/>
-        <c:crosses val="autoZero"/>
+        <c:crossesAt val="40544"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
@@ -4191,7 +4130,7 @@
       </c:spPr>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="b"/>
+      <c:legendPos val="t"/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -4205,16 +4144,13 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="50000"/>
-                  <a:lumOff val="50000"/>
-                </a:schemeClr>
+                <a:sysClr val="windowText" lastClr="000000"/>
               </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
             </a:defRPr>
           </a:pPr>
           <a:endParaRPr lang="en-US"/>
@@ -4252,7 +4188,13 @@
     <a:lstStyle/>
     <a:p>
       <a:pPr>
-        <a:defRPr/>
+        <a:defRPr sz="1200">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+          <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+          <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+        </a:defRPr>
       </a:pPr>
       <a:endParaRPr lang="en-US"/>
     </a:p>
@@ -13447,41 +13389,28 @@
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="20">
+  <a:schemeClr val="dk1"/>
   <cs:variation>
-    <a:lumMod val="60000"/>
+    <a:tint val="88500"/>
   </cs:variation>
   <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
+    <a:tint val="55000"/>
   </cs:variation>
   <cs:variation>
-    <a:lumMod val="80000"/>
+    <a:tint val="75000"/>
   </cs:variation>
   <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
+    <a:tint val="98500"/>
   </cs:variation>
   <cs:variation>
-    <a:lumMod val="50000"/>
+    <a:tint val="30000"/>
   </cs:variation>
   <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
+    <a:tint val="60000"/>
   </cs:variation>
   <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
+    <a:tint val="80000"/>
   </cs:variation>
 </cs:colorStyle>
 </file>
@@ -13607,18 +13536,18 @@
 </file>
 
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="280">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="276">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200" cap="all"/>
+    <cs:defRPr sz="1000" kern="1200"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -13626,8 +13555,8 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
@@ -13648,7 +13577,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
@@ -13664,7 +13593,7 @@
         <a:round/>
       </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
+    <cs:defRPr sz="1000" kern="1200"/>
   </cs:chartArea>
   <cs:dataLabel>
     <cs:lnRef idx="0"/>
@@ -13672,8 +13601,8 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -13707,62 +13636,36 @@
     </cs:bodyPr>
   </cs:dataLabelCallout>
   <cs:dataPoint>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="2">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="1"/>
+    <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:shade val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
   </cs:dataPoint>
   <cs:dataPoint3D>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="2">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="1"/>
+    <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:shade val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="2">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="1"/>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="15875" cap="rnd">
+      <a:ln w="28575" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
@@ -13774,33 +13677,30 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="2">
+    <cs:fillRef idx="1">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="1"/>
+    <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:shade val="95000"/>
-          </a:schemeClr>
+          <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="4"/>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
   <cs:dataPointWireframe>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="2"/>
+    <cs:fillRef idx="1"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="rnd">
@@ -13817,18 +13717,20 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
             <a:lumMod val="15000"/>
             <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
@@ -13838,7 +13740,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
@@ -13847,13 +13749,14 @@
           <a:lumOff val="25000"/>
         </a:schemeClr>
       </a:solidFill>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:downBar>
@@ -13862,17 +13765,17 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
             <a:lumMod val="35000"/>
             <a:lumOff val="65000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:prstDash val="dash"/>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:dropLine>
@@ -13881,16 +13784,17 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:errorBar>
@@ -13899,15 +13803,26 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
   </cs:floor>
   <cs:gridlineMajor>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
@@ -13926,16 +13841,17 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
             <a:lumMod val="5000"/>
             <a:lumOff val="95000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:gridlineMinor>
@@ -13944,17 +13860,17 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
             <a:lumMod val="50000"/>
             <a:lumOff val="50000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:prstDash val="dash"/>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:hiLoLine>
@@ -13963,16 +13879,17 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
             <a:lumMod val="35000"/>
             <a:lumOff val="65000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:leaderLine>
@@ -13982,8 +13899,8 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -13993,7 +13910,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
   </cs:plotArea>
   <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
@@ -14001,7 +13918,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
   </cs:plotArea3D>
   <cs:seriesAxis>
@@ -14010,8 +13927,8 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
@@ -14032,17 +13949,17 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
             <a:lumMod val="35000"/>
             <a:lumOff val="65000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:prstDash val="dash"/>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:seriesLine>
@@ -14052,26 +13969,27 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1400" kern="1200" cap="none" spc="20" baseline="0"/>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
   </cs:title>
   <cs:trendline>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="2"/>
+    <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="rnd">
+      <a:ln w="19050" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:prstDash val="sysDot"/>
       </a:ln>
     </cs:spPr>
   </cs:trendline>
@@ -14081,8 +13999,8 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -14092,19 +14010,20 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -14114,8 +14033,8 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -14125,8 +14044,14 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
   </cs:wall>
 </cs:chartStyle>
 </file>
@@ -15693,15 +15618,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>26</xdr:col>
-      <xdr:colOff>514350</xdr:colOff>
+      <xdr:colOff>438150</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>36</xdr:col>
-      <xdr:colOff>428625</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -15806,16 +15731,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>523875</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>90487</xdr:rowOff>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>176212</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>35</xdr:col>
-      <xdr:colOff>219075</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>166687</xdr:rowOff>
+      <xdr:col>44</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>61912</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -16160,13 +16085,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE2A62A6-3D73-4CE5-ABB5-A10C35402FCA}">
-  <dimension ref="A1:Z174"/>
+  <dimension ref="A1:AE174"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -16245,8 +16170,17 @@
       <c r="Z1" t="s">
         <v>25</v>
       </c>
+      <c r="AC1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>28</v>
+      </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>40544</v>
       </c>
@@ -16314,7 +16248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>40605</v>
       </c>
@@ -16370,7 +16304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>40617</v>
       </c>
@@ -16426,7 +16360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>40635</v>
       </c>
@@ -16482,7 +16416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>40638</v>
       </c>
@@ -16538,7 +16472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>40667</v>
       </c>
@@ -16618,7 +16552,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>40672</v>
       </c>
@@ -16674,7 +16608,7 @@
         <v>21.125</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>40679</v>
       </c>
@@ -16718,7 +16652,7 @@
         <v>21.125</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>40717</v>
       </c>
@@ -16798,7 +16732,7 @@
         <v>24.375</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>40721</v>
       </c>
@@ -16878,7 +16812,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>40862</v>
       </c>
@@ -16958,7 +16892,7 @@
         <v>45.5</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>40876</v>
       </c>
@@ -17038,7 +16972,7 @@
         <v>76.212500000000006</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>40877</v>
       </c>
@@ -17094,7 +17028,7 @@
         <v>76.212500000000006</v>
       </c>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>40973</v>
       </c>
@@ -17150,7 +17084,7 @@
         <v>76.212500000000006</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>40976</v>
       </c>

</xml_diff>

<commit_message>
updated version docs and added 2p1 convergence dashboard
</commit_message>
<xml_diff>
--- a/out/stir_daily_system_wide_with GRAPHS_22Oct25.xlsx
+++ b/out/stir_daily_system_wide_with GRAPHS_22Oct25.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c7d62234183fd3ba/Documents/GitHub/kerbel-long-term-impacts/out/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="8_{3109FC4A-BD15-44FB-B1BB-C01FAB71276C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{661B7CAB-B345-4CAE-AAAE-F088D9D70E99}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="8_{3109FC4A-BD15-44FB-B1BB-C01FAB71276C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B6D3ADC-6A4D-4687-820C-D8E0B88C8291}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{95A4D3B7-9F89-4514-B226-E93CDF5B25B1}"/>
+    <workbookView xWindow="-19305" yWindow="90" windowWidth="19410" windowHeight="20985" xr2:uid="{95A4D3B7-9F89-4514-B226-E93CDF5B25B1}"/>
   </bookViews>
   <sheets>
     <sheet name="stir_daily_system_wide" sheetId="1" r:id="rId1"/>

</xml_diff>